<commit_message>
fix spritesheet issue, 1-1 balancing, orc col vars
</commit_message>
<xml_diff>
--- a/docs/balancing.xlsx
+++ b/docs/balancing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5158e6b991fee7f4/Desktop/Schule/Maturarbeit/Godot/matura-roguelite/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="652" documentId="8_{1C25F502-3DF3-4C0E-A964-DFE0638285DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A209D46-F19E-44E5-A108-73993082925F}"/>
+  <xr:revisionPtr revIDLastSave="672" documentId="8_{1C25F502-3DF3-4C0E-A964-DFE0638285DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F69CE301-ECCB-445F-A0C6-1936876F7E08}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{5B9A7CE5-9E71-472F-BCC2-975C4625B76B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{5B9A7CE5-9E71-472F-BCC2-975C4625B76B}"/>
   </bookViews>
   <sheets>
     <sheet name="Room Balance" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Run Economy" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="218">
   <si>
     <t>Stage</t>
   </si>
@@ -132,12 +133,6 @@
     <t>Speed</t>
   </si>
   <si>
-    <t>Melee Range</t>
-  </si>
-  <si>
-    <t>Cooldown</t>
-  </si>
-  <si>
     <t>Knockback</t>
   </si>
   <si>
@@ -255,12 +250,6 @@
     <t>Slowness I</t>
   </si>
   <si>
-    <t>Player base speed gets slowed</t>
-  </si>
-  <si>
-    <t>Player base dmg reduction</t>
-  </si>
-  <si>
     <t>Damage reduction I</t>
   </si>
   <si>
@@ -270,12 +259,6 @@
     <t>More enemies</t>
   </si>
   <si>
-    <t>Enemies get HP boost</t>
-  </si>
-  <si>
-    <t>Stage 2</t>
-  </si>
-  <si>
     <t>Stage 3</t>
   </si>
   <si>
@@ -285,54 +268,12 @@
     <t>Weapon restriction</t>
   </si>
   <si>
-    <t>Player can't use current weapon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stage 3 </t>
-  </si>
-  <si>
-    <t>Only possible if enemy has more than 1 weapon unlocked</t>
-  </si>
-  <si>
     <t>Projectile speed boost</t>
   </si>
   <si>
-    <t>Enemy projectile speed gets buffed</t>
-  </si>
-  <si>
-    <t>Stage3</t>
-  </si>
-  <si>
-    <t>Only possible if one enemy type is ranged</t>
-  </si>
-  <si>
-    <t>Enemies melee range gets buffed</t>
-  </si>
-  <si>
     <t>Enemy range boost I</t>
   </si>
   <si>
-    <t xml:space="preserve">Restricted vision I </t>
-  </si>
-  <si>
-    <t>Player can't see outside of circle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Damage tick I </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Player takes constant damage </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enemy heal I </t>
-  </si>
-  <si>
-    <t>Enemy constantly heals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stage 1 </t>
-  </si>
-  <si>
     <t>Gold</t>
   </si>
   <si>
@@ -384,20 +325,389 @@
     <t>Training Dummy 2</t>
   </si>
   <si>
-    <t>1,1</t>
-  </si>
-  <si>
     <t>Enemy Difficulty</t>
   </si>
   <si>
     <t>training_dummy_2</t>
+  </si>
+  <si>
+    <t>Difficulty tier</t>
+  </si>
+  <si>
+    <t>Room-clear essence</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>enemy_health</t>
+  </si>
+  <si>
+    <t>Increase enemy maximum HP</t>
+  </si>
+  <si>
+    <t>Initial enemies in this room only.</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>more_enemies</t>
+  </si>
+  <si>
+    <t>Increase initial enemy count</t>
+  </si>
+  <si>
+    <t>Round extra count upward; use the room roster.</t>
+  </si>
+  <si>
+    <t>projectile_speed</t>
+  </si>
+  <si>
+    <t>Increase enemy projectile speed</t>
+  </si>
+  <si>
+    <t>Only eligible with projectile enemies.</t>
+  </si>
+  <si>
+    <t>melee_reach</t>
+  </si>
+  <si>
+    <t>Increase enemy melee reach</t>
+  </si>
+  <si>
+    <t>Only eligible with suitable melee enemies; attack visuals must match.</t>
+  </si>
+  <si>
+    <t>enemy_regeneration</t>
+  </si>
+  <si>
+    <t>Enemy heal I</t>
+  </si>
+  <si>
+    <t>Regenerate enemy maximum HP per second</t>
+  </si>
+  <si>
+    <t>Starts after 3 s without damage; fractional healing; never revive.</t>
+  </si>
+  <si>
+    <t>Deferred</t>
+  </si>
+  <si>
+    <t>slowness</t>
+  </si>
+  <si>
+    <t>Reduce player walking speed</t>
+  </si>
+  <si>
+    <t>Dash speed unchanged.</t>
+  </si>
+  <si>
+    <t>damage_reduction</t>
+  </si>
+  <si>
+    <t>Reduce player outgoing attack damage</t>
+  </si>
+  <si>
+    <t>Applies to player attacks in this room only.</t>
+  </si>
+  <si>
+    <t>restricted_vision</t>
+  </si>
+  <si>
+    <t>Restricted vision I</t>
+  </si>
+  <si>
+    <t>Limit vision to a 135 px radius</t>
+  </si>
+  <si>
+    <t>Logical pixels, not a percentage; soft edge; HUD remains visible. Playtest radius.</t>
+  </si>
+  <si>
+    <t>weapon_restriction</t>
+  </si>
+  <si>
+    <t>Disable current weapon (deferred)</t>
+  </si>
+  <si>
+    <t>Only if PLAYER owns another usable weapon; switching rules undecided.</t>
+  </si>
+  <si>
+    <t>enemy_haste</t>
+  </si>
+  <si>
+    <t>Enemy haste</t>
+  </si>
+  <si>
+    <t>Increase enemy walking / chase speed</t>
+  </si>
+  <si>
+    <t>Attack timings unchanged.</t>
+  </si>
+  <si>
+    <t>slow_recovery</t>
+  </si>
+  <si>
+    <t>Slow recovery</t>
+  </si>
+  <si>
+    <t>Reduce player stamina regeneration</t>
+  </si>
+  <si>
+    <t>Includes stamina-potion regeneration boost.</t>
+  </si>
+  <si>
+    <t>elite_defender</t>
+  </si>
+  <si>
+    <t>Elite defender</t>
+  </si>
+  <si>
+    <t>One marked enemy: +50% HP, +20% damage</t>
+  </si>
+  <si>
+    <t>Enemy Buff column is HP increase; damage increase is 20%.</t>
+  </si>
+  <si>
+    <t>reinforcements</t>
+  </si>
+  <si>
+    <t>Reinforcements</t>
+  </si>
+  <si>
+    <t>Add a wave after initial group dies</t>
+  </si>
+  <si>
+    <t>Extra count = ceil(initial count x 0.5); same roster; 1 s spawn warning.</t>
+  </si>
+  <si>
+    <t>Speed (px/s)</t>
+  </si>
+  <si>
+    <t>Hit radius (px)</t>
+  </si>
+  <si>
+    <t>Recovery (s)</t>
+  </si>
+  <si>
+    <t>Hit knockback (px/s)</t>
+  </si>
+  <si>
+    <t>1-1</t>
+  </si>
+  <si>
+    <t>Current scene values. Trigger range 25 px; windup 0.5 s, dash 100 px/s up to 0.3 s, spin 3 s. First-run 1-1 roster.</t>
+  </si>
+  <si>
+    <t>goblin_barrel</t>
+  </si>
+  <si>
+    <t>Goblin Barrel</t>
+  </si>
+  <si>
+    <t>1-1 replay</t>
+  </si>
+  <si>
+    <t>Current scene + hitbox defaults. Added after recorded 1-1 clear; also boss summons. Windup 0.18 s, dash 75 px/s for 0.5 s, swing 0.32 s; hit at 0.12 s.</t>
+  </si>
+  <si>
+    <t>green_goblin</t>
+  </si>
+  <si>
+    <t>Green Goblin</t>
+  </si>
+  <si>
+    <t>1-2</t>
+  </si>
+  <si>
+    <t>Implemented. Barrel-style attack; trigger 25 px, detection 80 px. Windup 0.18 s, dash 0.5 s, swing 0.32 s, hit at 0.12 s.</t>
+  </si>
+  <si>
+    <t>green_orc_archer</t>
+  </si>
+  <si>
+    <t>Green Orc Archer</t>
+  </si>
+  <si>
+    <t>Implemented; orc_archer is the 1-3 catalogue alias for this scene. Detection 160 px, fire range 100 px. Windup 0.18 s, attack 0.32 s, release at 0.12 s; arrow 180 px/s, lifetime 2 s.</t>
+  </si>
+  <si>
+    <t>orc_barbare</t>
+  </si>
+  <si>
+    <t>Green Orc Barbare</t>
+  </si>
+  <si>
+    <t>1-3</t>
+  </si>
+  <si>
+    <t>Implemented. Stationary swing, no dash. Trigger 25 px; windup 0.18 s, attack 0.32 s, hit at 0.12 s.</t>
+  </si>
+  <si>
+    <t>blue_orc_archer</t>
+  </si>
+  <si>
+    <t>Blue Orc Archer</t>
+  </si>
+  <si>
+    <t>Implemented. Same initial stats and size as green archer; tune separately later.</t>
+  </si>
+  <si>
+    <t>red_orc_archer</t>
+  </si>
+  <si>
+    <t>Red Orc Archer</t>
+  </si>
+  <si>
+    <t>blue_orc_barbare</t>
+  </si>
+  <si>
+    <t>Blue Orc Barbare</t>
+  </si>
+  <si>
+    <t>Implemented. Same initial stats and size as green Barbare; tune separately later.</t>
+  </si>
+  <si>
+    <t>red_orc_barbare</t>
+  </si>
+  <si>
+    <t>Red Orc Barbare</t>
+  </si>
+  <si>
+    <t>monster_slasher</t>
+  </si>
+  <si>
+    <t>MonsterSlasher</t>
+  </si>
+  <si>
+    <t>1-3 boss support</t>
+  </si>
+  <si>
+    <t>Implemented. Two opposite horizontal passes; dash 75 px/s, pass duration 0.5 s. Two initially; two more after goblin waves 1 and 2.</t>
+  </si>
+  <si>
+    <t>sorcerer</t>
+  </si>
+  <si>
+    <t>Sorcerer</t>
+  </si>
+  <si>
+    <t>1-3 boss</t>
+  </si>
+  <si>
+    <t>Implemented; stationary, summon-only (configured unused damage 5). First summon after 3 s; 3 waves of 3 barrels. Next wave waits for goblins to die. All support must die to clear.</t>
+  </si>
+  <si>
+    <t>frog_monster</t>
+  </si>
+  <si>
+    <t>FrogMonster</t>
+  </si>
+  <si>
+    <t>2-1; 2-3</t>
+  </si>
+  <si>
+    <t>Planned only. Melee; exact attack design and stats require approval.</t>
+  </si>
+  <si>
+    <t>mushroom</t>
+  </si>
+  <si>
+    <t>Mushroom</t>
+  </si>
+  <si>
+    <t>2-1; 2-2; 2-3</t>
+  </si>
+  <si>
+    <t>Planned only. Ranged; exact attack design and stats require approval.</t>
+  </si>
+  <si>
+    <t>ent</t>
+  </si>
+  <si>
+    <t>Ent</t>
+  </si>
+  <si>
+    <t>2-2; 2-3</t>
+  </si>
+  <si>
+    <t>cyclop_archer</t>
+  </si>
+  <si>
+    <t>Cyclop Archer</t>
+  </si>
+  <si>
+    <t>2-3</t>
+  </si>
+  <si>
+    <t>frog_boss</t>
+  </si>
+  <si>
+    <t>FrogBoss</t>
+  </si>
+  <si>
+    <t>2-3 boss</t>
+  </si>
+  <si>
+    <t>Planned only. Major boss; exact attack design and stats require approval.</t>
+  </si>
+  <si>
+    <t>dwarfette</t>
+  </si>
+  <si>
+    <t>Dwarfette / Wrecking Ball</t>
+  </si>
+  <si>
+    <t>3-1; 3-3</t>
+  </si>
+  <si>
+    <t>monsterfly</t>
+  </si>
+  <si>
+    <t>Monsterfly</t>
+  </si>
+  <si>
+    <t>3-1</t>
+  </si>
+  <si>
+    <t>Planned only. Regular enemy; exact attack design and stats require approval.</t>
+  </si>
+  <si>
+    <t>rhino_monster</t>
+  </si>
+  <si>
+    <t>RhinoMonster</t>
+  </si>
+  <si>
+    <t>Planned only. Charge enemy; formerly called Smasher; exact attack design and stats require approval.</t>
+  </si>
+  <si>
+    <t>vampire_archer</t>
+  </si>
+  <si>
+    <t>Vampire Archer</t>
+  </si>
+  <si>
+    <t>game_master</t>
+  </si>
+  <si>
+    <t>GameMaster</t>
+  </si>
+  <si>
+    <t>3-3 boss</t>
+  </si>
+  <si>
+    <t>1-2, 1-3</t>
+  </si>
+  <si>
+    <t>3-2, 3-3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -405,16 +715,316 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -422,25 +1032,225 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="42">
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
-      <protection locked="0" hidden="0"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -455,12 +1265,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{57CB6469-E74F-4269-A346-50BFACE0657B}" name="Table2" displayName="Table2" ref="A1:K37" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{57CB6469-E74F-4269-A346-50BFACE0657B}" name="Table2" displayName="Table2" ref="A1:K37" totalsRowShown="0">
   <autoFilter ref="A1:K37" xr:uid="{57CB6469-E74F-4269-A346-50BFACE0657B}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{01D57AB7-F17B-482F-8E6E-5C45BD970849}" name="Stage"/>
@@ -500,22 +1306,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{70DFE4FB-C52E-4503-98FE-26910E3BE33A}" name="Table4" displayName="Table4" ref="A1:M12" totalsRowShown="0">
-  <autoFilter ref="A1:M12" xr:uid="{70DFE4FB-C52E-4503-98FE-26910E3BE33A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FB41B092-5EB1-4212-B9E6-C0D670B06C2F}" name="Table6" displayName="Table6" ref="A1:M27" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:M27" xr:uid="{FB41B092-5EB1-4212-B9E6-C0D670B06C2F}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{3ED3C414-F1C4-4AD4-A7FA-BB8D138E7123}" name="Enemy ID"/>
-    <tableColumn id="2" xr3:uid="{D73DAA81-A1EC-454E-854B-C7FFD9FD1C4E}" name="Enemy Name"/>
-    <tableColumn id="3" xr3:uid="{496A8861-C4E7-45C5-89AB-B152899B41EF}" name="Stage Availability"/>
-    <tableColumn id="4" xr3:uid="{88323C6A-99B9-42A2-BBFD-03EAAD0AC332}" name="Enemy Difficulty"/>
-    <tableColumn id="5" xr3:uid="{7D95ED4E-6317-43A2-91C4-CA4B2C1B711B}" name="HP"/>
-    <tableColumn id="6" xr3:uid="{18903491-4564-4F3A-97BC-081C3101E3C2}" name="Melee Dmg"/>
-    <tableColumn id="7" xr3:uid="{ADAE7DD1-3F8B-4EFB-A6AD-774455CA1396}" name="Range Dmg"/>
-    <tableColumn id="8" xr3:uid="{AB2BA7DA-4ED0-402C-BC7E-C94098BBEB93}" name="Speed"/>
-    <tableColumn id="9" xr3:uid="{417E7893-83CF-454A-8B7C-7934FFF15B7C}" name="Melee Range"/>
-    <tableColumn id="10" xr3:uid="{887D4BBE-9B1B-458C-8487-927E7CEA2366}" name="Cooldown"/>
-    <tableColumn id="11" xr3:uid="{D3A26C2E-53B6-4630-80BA-B4F7965CA4A1}" name="Knockback"/>
-    <tableColumn id="12" xr3:uid="{72AE477C-C8C0-46FA-91D5-7C1B7B0CF024}" name="Weight"/>
-    <tableColumn id="13" xr3:uid="{A8809BD9-22AF-49D8-84E1-421E93C28FC2}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{46570C25-1084-4E9E-8948-80CCACEF9655}" name="Enemy ID"/>
+    <tableColumn id="2" xr3:uid="{50EE51A6-78D0-4A93-997A-C59B41904419}" name="Enemy Name"/>
+    <tableColumn id="3" xr3:uid="{6557213E-935C-49A8-B5B7-526A69D44FA4}" name="Stage Availability"/>
+    <tableColumn id="4" xr3:uid="{B5D3A691-70AA-42BA-AD52-274FDAEDE073}" name="Enemy Difficulty"/>
+    <tableColumn id="5" xr3:uid="{9EED8C32-74CC-4FC1-AD4A-CA184D2E5D44}" name="HP"/>
+    <tableColumn id="6" xr3:uid="{63F1D0CB-A151-4667-933C-97661FA9338C}" name="Melee Dmg"/>
+    <tableColumn id="7" xr3:uid="{C9F89C61-8892-4D9F-AD54-826E0BBDEF3B}" name="Range Dmg"/>
+    <tableColumn id="8" xr3:uid="{C6C027E3-4705-46A3-8234-DBBE1439D19C}" name="Speed (px/s)"/>
+    <tableColumn id="9" xr3:uid="{134AF165-8977-417F-B120-CA6D2329C024}" name="Hit radius (px)"/>
+    <tableColumn id="10" xr3:uid="{E0BDCC7C-2F70-489D-9E5D-B310C39B9714}" name="Recovery (s)"/>
+    <tableColumn id="11" xr3:uid="{4B847F7E-08E0-4AC1-9AA0-4074EDEDAF82}" name="Hit knockback (px/s)"/>
+    <tableColumn id="12" xr3:uid="{94294FDD-B23F-4A7F-A3FE-C2021A1EC0E8}" name="Weight"/>
+    <tableColumn id="13" xr3:uid="{1889C3B2-8F7C-4330-AC2A-88AF7B0FCCE2}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -542,22 +1348,23 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FB702AD7-4EAB-42E3-ABD7-1C4FD4B9D169}" name="Table6" displayName="Table6" ref="A1:J20" totalsRowShown="0">
-  <autoFilter ref="A1:J20" xr:uid="{FB702AD7-4EAB-42E3-ABD7-1C4FD4B9D169}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
-    <sortCondition ref="F1:F20"/>
-  </sortState>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{D8F8BBB6-BE1F-41FD-A8DC-455376D141AB}" name="Debuff ID"/>
-    <tableColumn id="2" xr3:uid="{589F47EA-2B36-4E22-8DF5-DA371CCDFF98}" name="Debuff Name"/>
-    <tableColumn id="3" xr3:uid="{F46F91B5-5FA1-41F4-9A37-F40B324E6F24}" name="Description"/>
-    <tableColumn id="4" xr3:uid="{6D2C7336-4153-4D97-AE8A-3FFF81472C3F}" name="Stage min"/>
-    <tableColumn id="5" xr3:uid="{BFD9232A-F2FC-4280-9876-344CF8F81E45}" name="Stage max"/>
-    <tableColumn id="6" xr3:uid="{410788DA-8813-4107-9FBE-54BB35F2E226}" name="Debuff % "/>
-    <tableColumn id="7" xr3:uid="{9BEE759F-4166-4BCE-87D8-EF160123EFBA}" name="Enemy Buff % "/>
-    <tableColumn id="8" xr3:uid="{F418EFE1-4BA3-412B-873C-4FC72B5D075B}" name="Difficulty"/>
-    <tableColumn id="9" xr3:uid="{7C59565E-0672-4F31-AA78-8349DD79EC74}" name="Weight"/>
-    <tableColumn id="10" xr3:uid="{300E5170-92DA-4591-94D7-D1158A71535A}" name="Notes"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{478591B9-48AC-4E58-889A-59E3D6CFAE54}" name="Table4" displayName="Table4" ref="A1:L14" totalsRowShown="0">
+  <autoFilter ref="A1:L14" xr:uid="{478591B9-48AC-4E58-889A-59E3D6CFAE54}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{2D48E5DA-F732-4E45-BC40-6061A538F167}" name="Debuff ID"/>
+    <tableColumn id="2" xr3:uid="{A2D16444-181E-4DA5-A9E6-5AF8816A3BCD}" name="Debuff Name"/>
+    <tableColumn id="3" xr3:uid="{5947692A-C4EB-4CA4-8045-12D99E402F71}" name="Description"/>
+    <tableColumn id="4" xr3:uid="{45CC64EE-850F-4E2F-980A-657BB3CD65E4}" name="Stage min"/>
+    <tableColumn id="5" xr3:uid="{71B20680-F3AC-4120-94C7-511288FDAFA2}" name="Stage max"/>
+    <tableColumn id="6" xr3:uid="{418120AD-AA5A-48AB-A24B-6393A8C37BD9}" name="Debuff % "/>
+    <tableColumn id="7" xr3:uid="{4C1C6E5F-ACCF-4739-8CB4-4DD02A4D1B5E}" name="Enemy Buff % "/>
+    <tableColumn id="8" xr3:uid="{A1F32C39-78DD-41E7-8BE6-A663CD74209A}" name="Difficulty tier"/>
+    <tableColumn id="9" xr3:uid="{D2F5C68C-452B-40E5-943B-88DCADDE0190}" name="Weight"/>
+    <tableColumn id="10" xr3:uid="{E41B4D2A-A03D-44B4-A104-6E40135EB1E2}" name="Notes"/>
+    <tableColumn id="11" xr3:uid="{165E848D-757A-4144-9089-4F77ADC5CB3B}" name="Room-clear essence">
+      <calculatedColumnFormula>IF(I2=0,0,H2)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{ED2A6768-0A09-4746-B2B4-B88ED8CA146D}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -990,38 +1797,38 @@
     <col min="11" max="11" width="49.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1120,7 +1927,7 @@
       <c r="I4">
         <v>0</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4">
         <v>0.2</v>
       </c>
     </row>
@@ -1152,7 +1959,7 @@
       <c r="I5">
         <v>6</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <v>0.1</v>
       </c>
       <c r="K5" t="s">
@@ -1248,7 +2055,7 @@
       <c r="I8">
         <v>0</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8">
         <v>0.2</v>
       </c>
     </row>
@@ -1280,7 +2087,7 @@
       <c r="I9">
         <v>8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9">
         <v>0.1</v>
       </c>
     </row>
@@ -1376,7 +2183,7 @@
       <c r="I12">
         <v>0</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12">
         <v>0.2</v>
       </c>
     </row>
@@ -1408,7 +2215,7 @@
       <c r="I13">
         <v>8</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13">
         <v>0.1</v>
       </c>
       <c r="K13" t="s">
@@ -1507,7 +2314,7 @@
       <c r="I16">
         <v>0</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16">
         <v>0.2</v>
       </c>
     </row>
@@ -1539,7 +2346,7 @@
       <c r="I17">
         <v>10</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17">
         <v>0.1</v>
       </c>
     </row>
@@ -1635,7 +2442,7 @@
       <c r="I20">
         <v>0</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20">
         <v>0.2</v>
       </c>
     </row>
@@ -1667,7 +2474,7 @@
       <c r="I21">
         <v>10</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21">
         <v>0.1</v>
       </c>
     </row>
@@ -1763,7 +2570,7 @@
       <c r="I24">
         <v>0</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24">
         <v>0.2</v>
       </c>
     </row>
@@ -1795,7 +2602,7 @@
       <c r="I25">
         <v>10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25">
         <v>0.1</v>
       </c>
       <c r="K25" t="s">
@@ -1894,7 +2701,7 @@
       <c r="I28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28">
         <v>0.2</v>
       </c>
     </row>
@@ -1926,7 +2733,7 @@
       <c r="I29">
         <v>12</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29">
         <v>0.1</v>
       </c>
     </row>
@@ -2022,7 +2829,7 @@
       <c r="I32">
         <v>0</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32">
         <v>0.2</v>
       </c>
     </row>
@@ -2054,7 +2861,7 @@
       <c r="I33">
         <v>15</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33">
         <v>0.1</v>
       </c>
     </row>
@@ -2153,7 +2960,7 @@
       <c r="I36">
         <v>0</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36">
         <v>0.35</v>
       </c>
     </row>
@@ -2185,7 +2992,7 @@
       <c r="I37">
         <v>30</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37">
         <v>0.15</v>
       </c>
       <c r="K37" t="s">
@@ -2201,99 +3008,595 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CEE3F12-2C6B-46B5-A814-8AFE08740C0E}">
-  <dimension ref="A1:M2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.90625" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="6.54296875" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" customWidth="1"/>
+    <col min="7" max="7" width="16.1796875" customWidth="1"/>
+    <col min="8" max="8" width="17.453125" customWidth="1"/>
+    <col min="9" max="9" width="19.453125" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="11.26953125" customWidth="1"/>
+    <col min="13" max="13" width="176.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="H1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K1" t="s">
-        <v>30</v>
-      </c>
-      <c r="L1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>112</v>
+        <v>91</v>
+      </c>
+      <c r="C2" t="s">
+        <v>148</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
+        <v>18</v>
+      </c>
+      <c r="I2">
+        <v>22</v>
+      </c>
+      <c r="J2">
+        <v>0.35</v>
+      </c>
+      <c r="K2">
+        <v>90</v>
+      </c>
+      <c r="M2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E3">
+        <v>16</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>40</v>
+      </c>
+      <c r="I3">
+        <v>20</v>
+      </c>
+      <c r="J3">
+        <v>0.8</v>
+      </c>
+      <c r="K3">
+        <v>180</v>
+      </c>
+      <c r="M3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4">
         <v>5</v>
       </c>
-      <c r="I2">
-        <v>14</v>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>40</v>
+      </c>
+      <c r="I4">
+        <v>20</v>
+      </c>
+      <c r="J4">
+        <v>0.8</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="M4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>40</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0.8</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="M5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C6" t="s">
+        <v>163</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>40</v>
+      </c>
+      <c r="I6">
+        <v>20</v>
+      </c>
+      <c r="J6">
+        <v>0.8</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="M6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" t="s">
+        <v>163</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>40</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0.8</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="M7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" t="s">
+        <v>169</v>
+      </c>
+      <c r="C8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="H8">
+        <v>40</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0.8</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="M8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" t="s">
+        <v>171</v>
+      </c>
+      <c r="C9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E9">
+        <v>20</v>
+      </c>
+      <c r="F9">
+        <v>5</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>40</v>
+      </c>
+      <c r="I9">
+        <v>20</v>
+      </c>
+      <c r="J9">
+        <v>0.8</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="M9" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>40</v>
+      </c>
+      <c r="I10">
+        <v>20</v>
+      </c>
+      <c r="J10">
+        <v>0.8</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="M10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>175</v>
+      </c>
+      <c r="B11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C11" t="s">
+        <v>177</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>5</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>40</v>
+      </c>
+      <c r="I11">
+        <v>20</v>
+      </c>
+      <c r="J11">
+        <v>0.8</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="M11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" t="s">
+        <v>181</v>
+      </c>
+      <c r="E12">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>120</v>
+      </c>
+      <c r="M12" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>183</v>
+      </c>
+      <c r="B13" t="s">
+        <v>184</v>
+      </c>
+      <c r="C13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M13" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" t="s">
+        <v>188</v>
+      </c>
+      <c r="C14" t="s">
+        <v>189</v>
+      </c>
+      <c r="M14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" t="s">
+        <v>192</v>
+      </c>
+      <c r="C15" t="s">
+        <v>193</v>
+      </c>
+      <c r="M15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>194</v>
+      </c>
+      <c r="B16" t="s">
+        <v>195</v>
+      </c>
+      <c r="C16" t="s">
+        <v>196</v>
+      </c>
+      <c r="M16" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" t="s">
+        <v>198</v>
+      </c>
+      <c r="C17" t="s">
+        <v>199</v>
+      </c>
+      <c r="M17" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>201</v>
+      </c>
+      <c r="B18" t="s">
+        <v>202</v>
+      </c>
+      <c r="C18" t="s">
+        <v>203</v>
+      </c>
+      <c r="M18" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>204</v>
+      </c>
+      <c r="B19" t="s">
+        <v>205</v>
+      </c>
+      <c r="C19" t="s">
+        <v>206</v>
+      </c>
+      <c r="M19" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>208</v>
+      </c>
+      <c r="B20" t="s">
+        <v>209</v>
+      </c>
+      <c r="C20" t="s">
+        <v>217</v>
+      </c>
+      <c r="M20" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" t="s">
+        <v>212</v>
+      </c>
+      <c r="C21" t="s">
+        <v>217</v>
+      </c>
+      <c r="M21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" t="s">
+        <v>214</v>
+      </c>
+      <c r="C22" t="s">
+        <v>215</v>
+      </c>
+      <c r="M22" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2318,34 +3621,34 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>38</v>
-      </c>
-      <c r="I1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J1" t="s">
-        <v>40</v>
       </c>
       <c r="K1" t="s">
         <v>10</v>
@@ -2360,290 +3663,611 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{017E2A2A-2DDA-4C5C-9A25-77F5430F61FC}">
-  <dimension ref="A1:J11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.7265625" customWidth="1"/>
     <col min="5" max="5" width="11.08984375" customWidth="1"/>
     <col min="6" max="6" width="10.453125" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="10" max="10" width="47" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.90625" customWidth="1"/>
+    <col min="8" max="8" width="13.36328125" customWidth="1"/>
+    <col min="9" max="9" width="8.6328125" customWidth="1"/>
+    <col min="10" max="10" width="67.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.36328125" customWidth="1"/>
+    <col min="12" max="12" width="8.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
         <v>41</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>42</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>43</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>44</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>45</v>
       </c>
-      <c r="F1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G1" t="s">
-        <v>47</v>
-      </c>
       <c r="H1" t="s">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="I1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>97</v>
+      </c>
       <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0.3</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>99</v>
+      </c>
+      <c r="K2">
+        <f t="shared" ref="K2:K6" si="0">IF(I2=0,0,H2)</f>
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0.4</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K3">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="L3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0.25</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="L4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0.2</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>109</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="L5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0.02</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>113</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="L6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>0.15</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>117</v>
+      </c>
+      <c r="K7">
+        <f>IF(I7=0,0,H7)</f>
+        <v>2</v>
+      </c>
+      <c r="L7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>0.2</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
+        <v>120</v>
+      </c>
+      <c r="K8">
+        <f>IF(I8=0,0,H8)</f>
+        <v>1</v>
+      </c>
+      <c r="L8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>2</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>124</v>
+      </c>
+      <c r="K9">
+        <f>IF(I9=0,0,H9)</f>
+        <v>2</v>
+      </c>
+      <c r="L9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" t="s">
         <v>72</v>
       </c>
-      <c r="C2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
+      <c r="C10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s">
+        <v>127</v>
+      </c>
+      <c r="K10">
+        <f>IF(I10=0,0,H10)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0.15</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11" t="s">
+        <v>131</v>
+      </c>
+      <c r="K11">
+        <f>IF(I11=0,0,H11)</f>
+        <v>1</v>
+      </c>
+      <c r="L11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>0.25</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>135</v>
+      </c>
+      <c r="K12">
+        <f>IF(I12=0,0,H12)</f>
+        <v>2</v>
+      </c>
+      <c r="L12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
         <v>0.5</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13" t="s">
+        <v>139</v>
+      </c>
+      <c r="K13">
+        <f>IF(I13=0,0,H13)</f>
+        <v>2</v>
+      </c>
+      <c r="L13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>140</v>
+      </c>
+      <c r="B14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" t="s">
-        <v>77</v>
-      </c>
-      <c r="E3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="H3" s="1">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="J4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" t="s">
-        <v>76</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>88</v>
-      </c>
-      <c r="C10" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F11" s="1">
-        <v>1</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0</v>
-      </c>
-      <c r="H11" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="J11" t="s">
-        <v>81</v>
-      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14" t="s">
+        <v>143</v>
+      </c>
+      <c r="K14">
+        <f>IF(I14=0,0,H14)</f>
+        <v>3</v>
+      </c>
+      <c r="L14" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A20:L20"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -2668,37 +4292,37 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" t="s">
         <v>43</v>
-      </c>
-      <c r="D1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" t="s">
-        <v>55</v>
-      </c>
-      <c r="I1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" t="s">
-        <v>45</v>
       </c>
       <c r="L1" t="s">
         <v>10</v>
@@ -2706,80 +4330,80 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="K2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="H3">
         <v>8</v>
       </c>
       <c r="J3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="K3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="F4">
         <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="H4">
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="K4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2830,100 +4454,100 @@
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" t="s">
         <v>58</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>59</v>
       </c>
-      <c r="F1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" t="s">
         <v>60</v>
-      </c>
-      <c r="H1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J1" t="s">
-        <v>62</v>
       </c>
       <c r="K1" t="s">
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="M1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O1" t="s">
         <v>56</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>57</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R1" t="s">
         <v>58</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" t="s">
-        <v>43</v>
-      </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
+        <v>50</v>
+      </c>
+      <c r="U1" t="s">
         <v>60</v>
-      </c>
-      <c r="S1" t="s">
-        <v>61</v>
-      </c>
-      <c r="T1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U1" t="s">
-        <v>62</v>
       </c>
       <c r="V1" t="s">
         <v>10</v>
       </c>
       <c r="W1" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="X1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z1" t="s">
         <v>56</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AA1" t="s">
         <v>57</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AB1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC1" t="s">
         <v>58</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AD1" t="s">
         <v>59</v>
       </c>
-      <c r="AB1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AC1" t="s">
+      <c r="AE1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF1" t="s">
         <v>60</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>62</v>
       </c>
       <c r="AG1" t="s">
         <v>10</v>
@@ -2931,34 +4555,34 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C43" t="s">
+        <v>55</v>
+      </c>
+      <c r="D43" t="s">
         <v>56</v>
       </c>
-      <c r="C43" t="s">
+      <c r="E43" t="s">
         <v>57</v>
       </c>
-      <c r="D43" t="s">
+      <c r="F43" t="s">
+        <v>41</v>
+      </c>
+      <c r="G43" t="s">
         <v>58</v>
       </c>
-      <c r="E43" t="s">
+      <c r="H43" t="s">
         <v>59</v>
       </c>
-      <c r="F43" t="s">
-        <v>43</v>
-      </c>
-      <c r="G43" t="s">
+      <c r="I43" t="s">
+        <v>50</v>
+      </c>
+      <c r="J43" t="s">
         <v>60</v>
-      </c>
-      <c r="H43" t="s">
-        <v>61</v>
-      </c>
-      <c r="I43" t="s">
-        <v>52</v>
-      </c>
-      <c r="J43" t="s">
-        <v>62</v>
       </c>
       <c r="K43" t="s">
         <v>10</v>
@@ -2989,34 +4613,34 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
         <v>63</v>
-      </c>
-      <c r="B1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>65</v>
       </c>
       <c r="E1" t="s">
         <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G1" t="s">
         <v>27</v>
       </c>
       <c r="H1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K1" t="s">
         <v>10</v>
@@ -3024,7 +4648,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>